<commit_message>
completed datasets for apr 2026  - ready for analysis
</commit_message>
<xml_diff>
--- a/saved_data/top_artist_africa_metrics_1_apr_2026.xlsx
+++ b/saved_data/top_artist_africa_metrics_1_apr_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Files\spotify_music_analysis\saved_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743358DD-F2A7-4028-A2CA-F10332D74AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8208DDC-444A-4D7E-AA41-37582E9885DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="436" xr2:uid="{0C2FF910-49ED-45FA-A23C-1D15CC9ADB7F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
   <si>
     <t>Country</t>
   </si>
@@ -151,6 +151,15 @@
   </si>
   <si>
     <t>Ethiopia</t>
+  </si>
+  <si>
+    <t>TikTok Followers</t>
+  </si>
+  <si>
+    <t>Instagram Followers</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -516,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{999CDD1F-9799-49A3-94B5-D8F2FCE0D205}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -527,9 +536,11 @@
     <col min="6" max="6" width="22.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" ht="14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="14" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -554,8 +565,14 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -580,8 +597,14 @@
       <c r="H2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2">
+        <v>253000</v>
+      </c>
+      <c r="J2">
+        <v>60400</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -606,8 +629,14 @@
       <c r="H3">
         <v>62</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3">
+        <v>2300000</v>
+      </c>
+      <c r="J3">
+        <v>7140000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -632,8 +661,14 @@
       <c r="H4">
         <v>163</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4">
+        <v>16200000</v>
+      </c>
+      <c r="J4">
+        <v>13600000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -658,8 +693,14 @@
       <c r="H5">
         <v>366</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5">
+        <v>290000</v>
+      </c>
+      <c r="J5">
+        <v>963000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -684,8 +725,14 @@
       <c r="H6">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6">
+        <v>12700000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -710,8 +757,14 @@
       <c r="H7">
         <v>106</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I7">
+        <v>1200000</v>
+      </c>
+      <c r="J7">
+        <v>8600000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -736,8 +789,14 @@
       <c r="H8">
         <v>160</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8">
+        <v>79700</v>
+      </c>
+      <c r="J8">
+        <v>213000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -762,8 +821,14 @@
       <c r="H9">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9">
+        <v>337000</v>
+      </c>
+      <c r="J9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -788,8 +853,14 @@
       <c r="H10">
         <v>81</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I10">
+        <v>1300000</v>
+      </c>
+      <c r="J10">
+        <v>4360000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -814,8 +885,14 @@
       <c r="H11">
         <v>202</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I11">
+        <v>133000</v>
+      </c>
+      <c r="J11">
+        <v>2060000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -840,8 +917,14 @@
       <c r="H12">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I12">
+        <v>16300</v>
+      </c>
+      <c r="J12">
+        <v>68900</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -866,8 +949,14 @@
       <c r="H13">
         <v>260</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I13">
+        <v>676000</v>
+      </c>
+      <c r="J13">
+        <v>351000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
@@ -892,8 +981,14 @@
       <c r="H14">
         <v>1566</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I14">
+        <v>10400000</v>
+      </c>
+      <c r="J14">
+        <v>19000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -918,8 +1013,14 @@
       <c r="H15">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15">
+        <v>5400000</v>
+      </c>
+      <c r="J15">
+        <v>910000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -944,8 +1045,14 @@
       <c r="H16">
         <v>372</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I16" t="s">
+        <v>44</v>
+      </c>
+      <c r="J16">
+        <v>525000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -970,8 +1077,14 @@
       <c r="H17">
         <v>283</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I17">
+        <v>5500000</v>
+      </c>
+      <c r="J17">
+        <v>6540000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
@@ -995,6 +1108,12 @@
       </c>
       <c r="H18">
         <v>5</v>
+      </c>
+      <c r="I18" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18">
+        <v>27700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>